<commit_message>
TRACKER v1.8: the two capital-call columns
The app reads Next call date and Next call amount, and the spreadsheet it handed you had
nowhere to write them. This template is maintained separately from the Exit Timing
Calendar's because it grows the You, Balances, Property, Cashflows and Events sheets the
retirement simulator needs, so the change to that one did not reach this one.

Optional, as before. Leave them blank and nothing changes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracker-template.xlsx
+++ b/tracker-template.xlsx
@@ -252,7 +252,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -414,6 +414,9 @@
     <xf numFmtId="167" fontId="18" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="18" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="18" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -810,13 +813,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A2:B49"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="24" min="1" max="1"/>
     <col width="104" customWidth="1" style="24" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="24.45" customHeight="1" s="25">
       <c r="B2" s="26" t="inlineStr">
         <is>
@@ -831,6 +835,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="17" customHeight="1" s="25">
       <c r="B5" s="28" t="inlineStr">
         <is>
@@ -845,6 +850,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="17" customHeight="1" s="25">
       <c r="B8" s="28" t="inlineStr">
         <is>
@@ -887,6 +893,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="17" customHeight="1" s="25">
       <c r="B15" s="28" t="inlineStr">
         <is>
@@ -936,141 +943,163 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="17" customHeight="1" s="25">
       <c r="B23" s="28" t="inlineStr">
         <is>
+          <t>If you know when your next capital call is due</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="25">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Fill in Next call date, and Next call amount if you know it. Any spelling of the date works (2027, Q1 2027, March 2027) because only the year is used. Leave them blank and the tool spreads whatever is still uncalled evenly over about three years from the year after you funded, which is what it has always done. An amount with no date cannot be placed in a year, so it is ignored and the tool says so.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1" s="25">
+      <c r="B25" s="28" t="inlineStr">
+        <is>
           <t>Cell colours</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="25">
-      <c r="B24" s="31" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">   Yellow fill  —  Fill this in.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="25">
-      <c r="B25" s="32" t="inlineStr">
+    <row r="27" ht="15" customHeight="1" s="25">
+      <c r="B27" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">   White  —  A formula. Leave it alone.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1" s="25">
-      <c r="B27" s="33" t="inlineStr">
+    <row r="28"/>
+    <row r="29">
+      <c r="B29" s="33" t="inlineStr">
         <is>
           <t>Not advice. The probability assumptions in the prompt are one investor’s and are meant to be argued with.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="24" t="inlineStr">
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="24" t="inlineStr">
         <is>
           <t>Deals in fund, Liquidity from, Liquidity to</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="24" t="inlineStr">
-        <is>
-          <t>How many underlying deals the position holds. This decides only how a VENTURE position is priced: a venture fund holding 20 or more is not priced like a single company. You do not need it for a fund that pays a coupon. Put 1 here if the position is a SINGLE COMPANY that pays a preferred return, which tells the tool to exit it on one date instead of spreading the payout.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="24" t="inlineStr">
         <is>
+          <t>How many underlying deals the position holds. This decides only how a VENTURE position is priced: a venture fund holding 20 or more is not priced like a single company. You do not need it for a fund that pays a coupon. Put 1 here if the position is a SINGLE COMPANY that pays a preferred return, which tells the tool to exit it on one date instead of spreading the payout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" s="24" t="inlineStr">
+        <is>
           <t>Liquidity from / Liquidity to</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="24" t="inlineStr">
-        <is>
-          <t>The years, counted from when you funded the deal, over which the fund actually sells down and pays out. If a sponsor has said "expect distributions in years five through eight", put 5 and 8. Leave them blank and the tool assumes the back 40% of the hold. Note that a pay-out window and a fund's stated life are not the same thing: a fund can finish selling in year six and wind up in year seven.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
+          <t>The years, counted from when you funded the deal, over which the fund actually sells down and pays out. If a sponsor has said "expect distributions in years five through eight", put 5 and 8. Leave them blank and the tool assumes the back 40% of the hold. Note that a pay-out window and a fund's stated life are not the same thing: a fund can finish selling in year six and wind up in year seven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="24" t="inlineStr">
+        <is>
           <t>You can leave most of this blank</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="24" t="inlineStr">
-        <is>
-          <t>The tool ships with a shared file for each of the common GC deals, carrying the sponsor, the vehicle, the structure, the preferred rate, the hold, the fees and when the GP says it pays out. If your deal name matches one of those, those columns fill themselves in and you only need YOUR numbers: commitment, funded to date, uncalled, and the year you funded it. Anything you do type wins over the shared file, always. A deal nobody has shared still works; you just supply its terms yourself.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="24" t="inlineStr">
         <is>
+          <t>The tool ships with a shared file for each of the common GC deals, carrying the sponsor, the vehicle, the structure, the preferred rate, the hold, the fees and when the GP says it pays out. If your deal name matches one of those, those columns fill themselves in and you only need YOUR numbers: commitment, funded to date, uncalled, and the year you funded it. Anything you do type wins over the shared file, always. A deal nobody has shared still works; you just supply its terms yourself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" s="24" t="inlineStr">
+        <is>
           <t>Thesis</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="24" t="inlineStr">
-        <is>
-          <t>Why you did the deal, in your own words. This is yours and it is never pre-filled from anywhere, because somebody else's reasoning is not your reasoning. It shows on the deal card and never leaves your machine.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="24" t="inlineStr">
         <is>
+          <t>Why you did the deal, in your own words. This is yours and it is never pre-filled from anywhere, because somebody else's reasoning is not your reasoning. It shows on the deal card and never leaves your machine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43">
+      <c r="A43" s="24" t="inlineStr">
+        <is>
           <t>Fund or Single deal</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="24" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="24" t="inlineStr">
         <is>
           <t>Type "Fund" if the position holds several underlying investments, or "Single deal" if it is one company or one property. This is the simplest way to tell the tool how a position pays out: a fund sells down over several years, a single deal is bought on one date. It beats anything the tool would otherwise guess, including the Deals in fund count. If you leave it blank the tool still works out a sensible answer, but saying it outright is better.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="51" t="inlineStr">
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" s="51" t="inlineStr">
         <is>
           <t>NEW IN THIS VERSION</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="52" t="inlineStr">
-        <is>
-          <t>· Account, on Positions: which account each deal is held in. Leave it blank and everything still works.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="52" t="inlineStr">
-        <is>
-          <t>· You: your ages, your spend target and your benefit. Drives the Liquidity Runway tab.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="52" t="inlineStr">
         <is>
-          <t>· Balances: everything that is not a private deal, one row per account and sleeve.</t>
+          <t>· Account, on Positions: which account each deal is held in. Leave it blank and everything still works.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="52" t="inlineStr">
         <is>
-          <t>· Property, Cashflows and Events: a house sale, a pension, an inheritance, a big bill.</t>
+          <t>· You: your ages, your spend target and your benefit. Drives the Liquidity Runway tab.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="52" t="inlineStr">
+        <is>
+          <t>· Balances: everything that is not a private deal, one row per account and sleeve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="52" t="inlineStr">
+        <is>
+          <t>· Property, Cashflows and Events: a house sale, a pension, an inheritance, a big bill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="52" t="inlineStr">
         <is>
           <t>· All three are optional. A tracker without them behaves exactly as it did before.</t>
         </is>
@@ -1089,7 +1118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:X21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="24" min="1" max="1"/>
@@ -1109,12 +1138,14 @@
     <col width="46" customWidth="1" style="25" min="19" max="19"/>
     <col width="18" customWidth="1" style="25" min="20" max="20"/>
     <col width="15" customWidth="1" style="25" min="21" max="21"/>
+    <col width="18" customWidth="1" style="25" min="23" max="23"/>
+    <col width="18" customWidth="1" style="25" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="16.15" customHeight="1" s="25">
       <c r="A1" s="34" t="inlineStr">
         <is>
-          <t>Positions  ·  fill in the yellow cells, one row per deal        TRACKER v1.7</t>
+          <t>Positions  ·  fill in the yellow cells, one row per deal        TRACKER v1.8</t>
         </is>
       </c>
     </row>
@@ -1227,6 +1258,16 @@
       <c r="V2" s="36" t="inlineStr">
         <is>
           <t>Marked Up MOIC</t>
+        </is>
+      </c>
+      <c r="W2" s="36" t="inlineStr">
+        <is>
+          <t>Next call date</t>
+        </is>
+      </c>
+      <c r="X2" s="36" t="inlineStr">
+        <is>
+          <t>Next call amount</t>
         </is>
       </c>
     </row>
@@ -1291,6 +1332,8 @@
       </c>
       <c r="U3" s="37" t="n"/>
       <c r="V3" s="42" t="n"/>
+      <c r="W3" s="59" t="n"/>
+      <c r="X3" s="37" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="25">
       <c r="A4" s="37" t="inlineStr">
@@ -1349,6 +1392,8 @@
       <c r="T4" s="37" t="n"/>
       <c r="U4" s="37" t="n"/>
       <c r="V4" s="42" t="n"/>
+      <c r="W4" s="59" t="n"/>
+      <c r="X4" s="37" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="25">
       <c r="A5" s="37" t="inlineStr">
@@ -1407,6 +1452,8 @@
       <c r="T5" s="37" t="n"/>
       <c r="U5" s="37" t="n"/>
       <c r="V5" s="42" t="n"/>
+      <c r="W5" s="59" t="n"/>
+      <c r="X5" s="37" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="25">
       <c r="A6" s="37" t="inlineStr">
@@ -1460,6 +1507,8 @@
       <c r="T6" s="37" t="n"/>
       <c r="U6" s="37" t="n"/>
       <c r="V6" s="42" t="n"/>
+      <c r="W6" s="59" t="n"/>
+      <c r="X6" s="37" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="25">
       <c r="A7" s="37" t="inlineStr">
@@ -1517,6 +1566,12 @@
       </c>
       <c r="U7" s="37" t="n"/>
       <c r="V7" s="42" t="n"/>
+      <c r="W7" s="59" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="X7" s="37" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="25">
       <c r="A8" s="37" t="inlineStr">
@@ -1574,6 +1629,8 @@
       </c>
       <c r="U8" s="37" t="n"/>
       <c r="V8" s="42" t="n"/>
+      <c r="W8" s="59" t="n"/>
+      <c r="X8" s="37" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="25">
       <c r="A9" s="37" t="inlineStr">
@@ -1627,6 +1684,8 @@
       <c r="T9" s="37" t="n"/>
       <c r="U9" s="37" t="n"/>
       <c r="V9" s="42" t="n"/>
+      <c r="W9" s="59" t="n"/>
+      <c r="X9" s="37" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="25">
       <c r="A10" s="37" t="inlineStr">
@@ -1680,6 +1739,8 @@
       <c r="T10" s="37" t="n"/>
       <c r="U10" s="37" t="n"/>
       <c r="V10" s="42" t="n"/>
+      <c r="W10" s="59" t="n"/>
+      <c r="X10" s="37" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="25">
       <c r="A11" s="37" t="inlineStr">
@@ -1733,6 +1794,8 @@
       <c r="T11" s="37" t="n"/>
       <c r="U11" s="37" t="n"/>
       <c r="V11" s="42" t="n"/>
+      <c r="W11" s="59" t="n"/>
+      <c r="X11" s="37" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="25">
       <c r="A12" s="37" t="inlineStr">
@@ -1786,6 +1849,8 @@
       <c r="T12" s="37" t="n"/>
       <c r="U12" s="37" t="n"/>
       <c r="V12" s="42" t="n"/>
+      <c r="W12" s="59" t="n"/>
+      <c r="X12" s="37" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
       <c r="A13" s="37" t="inlineStr">
@@ -1839,6 +1904,8 @@
       <c r="T13" s="37" t="n"/>
       <c r="U13" s="37" t="n"/>
       <c r="V13" s="42" t="n"/>
+      <c r="W13" s="59" t="n"/>
+      <c r="X13" s="37" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
       <c r="A14" s="37" t="inlineStr">
@@ -1892,6 +1959,8 @@
       <c r="T14" s="37" t="n"/>
       <c r="U14" s="37" t="n"/>
       <c r="V14" s="42" t="n"/>
+      <c r="W14" s="59" t="n"/>
+      <c r="X14" s="37" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
       <c r="A15" s="37" t="inlineStr">
@@ -1945,6 +2014,8 @@
       <c r="T15" s="37" t="n"/>
       <c r="U15" s="37" t="n"/>
       <c r="V15" s="42" t="n"/>
+      <c r="W15" s="59" t="n"/>
+      <c r="X15" s="37" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
       <c r="A16" s="46" t="inlineStr">
@@ -1973,8 +2044,13 @@
           <t>Single deal</t>
         </is>
       </c>
-    </row>
-    <row r="17"/>
+      <c r="W16" s="59" t="n"/>
+      <c r="X16" s="37" t="n"/>
+    </row>
+    <row r="17">
+      <c r="W17" s="59" t="n"/>
+      <c r="X17" s="37" t="n"/>
+    </row>
     <row r="18" ht="15" customHeight="1" s="25">
       <c r="A18" s="48" t="inlineStr">
         <is>
@@ -1992,6 +2068,8 @@
           <t>Single deal</t>
         </is>
       </c>
+      <c r="W18" s="59" t="n"/>
+      <c r="X18" s="37" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="24" t="inlineStr">
@@ -1999,6 +2077,8 @@
           <t>Hold, Coupon, Sponsor MOIC, Asset class and the fund columns are deliberately BLANK on these example rows. Those terms are identical for everyone who bought the deal, so they now live in one shared file per deal and the tool fills them in. Anything you type here overrides the shared file and nothing argues with you — which is why a figure typed before a sponsor corrected its terms is worth checking.</t>
         </is>
       </c>
+      <c r="W19" s="59" t="n"/>
+      <c r="X19" s="37" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="25">
       <c r="A20" s="48" t="inlineStr">
@@ -2017,6 +2097,8 @@
           <t>Single deal</t>
         </is>
       </c>
+      <c r="W20" s="59" t="n"/>
+      <c r="X20" s="37" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="24" t="inlineStr">
@@ -2024,6 +2106,8 @@
           <t>Marked Up MOIC is optional. It records what you believe a position is worth now, and it drives a paper track shown beside the cash forecast rather than inside it. It never moves a cash figure and never enters the IRR.</t>
         </is>
       </c>
+      <c r="W21" s="59" t="n"/>
+      <c r="X21" s="37" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>